<commit_message>
Se modifico la tabla de recoleccion de datos
</commit_message>
<xml_diff>
--- a/DiagramaDeGannt.xlsx
+++ b/DiagramaDeGannt.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia_4m9iwa1\Desktop\Julián\IUSH\Investigación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\OneDrive\Documentos\Competencias-Investigativas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140E5A83-0E8C-4818-B78E-1E5B5B385C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70946C1C-83B5-4642-B862-0073509A42F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Actividad</t>
   </si>
@@ -189,13 +189,28 @@
     <t>Escalas de medición</t>
   </si>
   <si>
-    <t>Censos</t>
-  </si>
-  <si>
     <t>Entrevista estructurada</t>
   </si>
   <si>
     <t>Estadística descriptiva</t>
+  </si>
+  <si>
+    <t>Observación directa, revisión documental</t>
+  </si>
+  <si>
+    <t>Análisis y validación experimental, métricas de desempeño</t>
+  </si>
+  <si>
+    <t>Evaluación funcional</t>
+  </si>
+  <si>
+    <t>Estadística inferencial, análisis de varianza</t>
+  </si>
+  <si>
+    <t>Informes técnicos, registros de pruebas</t>
+  </si>
+  <si>
+    <t>Bitácora técnica</t>
   </si>
 </sst>
 </file>
@@ -496,7 +511,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -515,105 +530,96 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -636,6 +642,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -684,7 +708,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2214,16 +2238,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
-    <col min="4" max="4" width="10.1796875" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="1" max="1" width="44.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="5" width="10.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>26</v>
       </c>
@@ -2240,7 +2263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -2258,7 +2281,7 @@
         <v>46098</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -2276,7 +2299,7 @@
         <v>46111</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>17</v>
       </c>
@@ -2294,7 +2317,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -2312,7 +2335,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
@@ -2330,7 +2353,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -2348,7 +2371,7 @@
         <v>46135</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -2366,7 +2389,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2384,7 +2407,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -2403,7 +2426,7 @@
       </c>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
@@ -2421,7 +2444,7 @@
         <v>46339</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -2439,7 +2462,7 @@
         <v>46563</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
         <v>27</v>
       </c>
@@ -2447,7 +2470,7 @@
         <v>46060</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
         <v>28</v>
       </c>
@@ -2455,7 +2478,7 @@
         <v>46362</v>
       </c>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D19" s="6"/>
     </row>
   </sheetData>
@@ -2471,185 +2494,195 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7D412B7-2AD2-4EEF-9661-1E8932A91675}">
   <dimension ref="B1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.36328125" customWidth="1"/>
-    <col min="2" max="2" width="12.90625" customWidth="1"/>
-    <col min="3" max="3" width="32.08984375" customWidth="1"/>
-    <col min="4" max="4" width="19.6328125" customWidth="1"/>
-    <col min="5" max="5" width="16.90625" customWidth="1"/>
+    <col min="1" max="1" width="3.33203125" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="32.109375" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B2" s="8" t="s">
+    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B2" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="11"/>
-    </row>
-    <row r="3" spans="2:8" ht="24.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="9"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="13"/>
-    </row>
-    <row r="4" spans="2:8" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="32" t="s">
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="31"/>
+    </row>
+    <row r="3" spans="2:8" ht="24.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="32"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="34"/>
+    </row>
+    <row r="4" spans="2:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="D4" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="19" t="s">
         <v>30</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="2:8" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="14" t="s">
+    <row r="5" spans="2:8" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="40" t="s">
         <v>51</v>
-      </c>
-      <c r="E5" s="43" t="s">
-        <v>52</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="2:8" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16"/>
-      <c r="C6" s="17" t="s">
+    <row r="6" spans="2:8" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="24"/>
+      <c r="C6" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" s="44"/>
+      <c r="D6" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="41"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="2:8" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="16"/>
-      <c r="C7" s="17" t="s">
+    <row r="7" spans="2:8" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="24"/>
+      <c r="C7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="44"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="41"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="2:8" ht="39.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="18"/>
-      <c r="C8" s="19" t="s">
+    <row r="8" spans="2:8" ht="39.450000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="25"/>
+      <c r="C8" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="45"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="42"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="2:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="20" t="s">
+    <row r="9" spans="2:8" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="35"/>
+      <c r="E9" s="49" t="s">
+        <v>53</v>
+      </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
     </row>
-    <row r="10" spans="2:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="22"/>
-      <c r="C10" s="23" t="s">
+    <row r="10" spans="2:8" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="27"/>
+      <c r="C10" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="47"/>
-      <c r="E10" s="36"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="50"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="2:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="22"/>
-      <c r="C11" s="23" t="s">
+    <row r="11" spans="2:8" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="27"/>
+      <c r="C11" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="47"/>
-      <c r="E11" s="36"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="50"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="2:8" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
+    <row r="12" spans="2:8" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="28"/>
+      <c r="C12" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="48"/>
-      <c r="E12" s="37"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="51"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="2:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="26" t="s">
+    <row r="13" spans="2:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="27"/>
-      <c r="E13" s="38"/>
+      <c r="D13" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>54</v>
+      </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="2:8" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="28"/>
-      <c r="C14" s="29" t="s">
+    <row r="14" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="36"/>
+      <c r="C14" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="39"/>
+      <c r="E14" s="21" t="s">
+        <v>55</v>
+      </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" spans="2:8" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="30"/>
-      <c r="C15" s="31" t="s">
+    <row r="15" spans="2:8" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="37"/>
+      <c r="C15" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="42"/>
-      <c r="E15" s="40"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="22" t="s">
+        <v>56</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2658,7 +2691,7 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -2667,7 +2700,7 @@
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -2676,7 +2709,7 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2685,7 +2718,7 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -2694,7 +2727,7 @@
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -2703,7 +2736,7 @@
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -2712,7 +2745,7 @@
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -2721,7 +2754,7 @@
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -2730,7 +2763,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -2739,7 +2772,7 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -2748,7 +2781,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -2757,7 +2790,7 @@
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -2766,7 +2799,7 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -2775,7 +2808,7 @@
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2784,7 +2817,7 @@
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -2793,7 +2826,7 @@
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -2802,7 +2835,7 @@
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -2811,7 +2844,7 @@
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -2820,7 +2853,7 @@
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -2829,7 +2862,7 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
@@ -2838,7 +2871,7 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -2848,7 +2881,7 @@
       <c r="H37" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="B5:B8"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="B2:E3"/>
@@ -2856,6 +2889,8 @@
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="E5:E8"/>
     <mergeCell ref="D9:D12"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E9:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Se actualiza formato, se completan las correcciones, se hace la ecucación de la muestra poblacional y se termina el marco teórico. Queda faltando hablar sobre el tipo de antena a utilizar y la caracterización dle material.
</commit_message>
<xml_diff>
--- a/DiagramaDeGannt.xlsx
+++ b/DiagramaDeGannt.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\OneDrive\Documentos\Competencias-Investigativas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia_4m9iwa1\Desktop\Julián\IUSH\Investigación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70946C1C-83B5-4642-B862-0073509A42F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C06DF48-777D-4603-82E5-343582A0C913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma" sheetId="1" r:id="rId1"/>
     <sheet name="Registro Resultados" sheetId="2" r:id="rId2"/>
+    <sheet name="Población" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>Actividad</t>
   </si>
@@ -211,6 +212,24 @@
   </si>
   <si>
     <t>Bitácora técnica</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>n</t>
   </si>
 </sst>
 </file>
@@ -708,7 +727,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2238,15 +2257,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="5" width="10.21875" customWidth="1"/>
+    <col min="1" max="1" width="44.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="4" max="5" width="10.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>26</v>
       </c>
@@ -2263,7 +2282,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -2281,7 +2300,7 @@
         <v>46098</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -2299,7 +2318,7 @@
         <v>46111</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>17</v>
       </c>
@@ -2317,7 +2336,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -2335,7 +2354,7 @@
         <v>46116</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
@@ -2353,7 +2372,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -2371,7 +2390,7 @@
         <v>46135</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -2389,7 +2408,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2407,7 +2426,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -2426,7 +2445,7 @@
       </c>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
@@ -2444,7 +2463,7 @@
         <v>46339</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -2462,7 +2481,7 @@
         <v>46563</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>27</v>
       </c>
@@ -2470,7 +2489,7 @@
         <v>46060</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
         <v>28</v>
       </c>
@@ -2478,7 +2497,7 @@
         <v>46362</v>
       </c>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D19" s="6"/>
     </row>
   </sheetData>
@@ -2494,17 +2513,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7D412B7-2AD2-4EEF-9661-1E8932A91675}">
   <dimension ref="B1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" customWidth="1"/>
-    <col min="2" max="2" width="12.88671875" customWidth="1"/>
-    <col min="3" max="3" width="32.109375" customWidth="1"/>
-    <col min="4" max="4" width="19.6640625" customWidth="1"/>
-    <col min="5" max="5" width="20.109375" customWidth="1"/>
+    <col min="1" max="1" width="3.36328125" customWidth="1"/>
+    <col min="2" max="2" width="12.90625" customWidth="1"/>
+    <col min="3" max="3" width="32.08984375" customWidth="1"/>
+    <col min="4" max="4" width="19.6328125" customWidth="1"/>
+    <col min="5" max="5" width="20.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B2" s="29" t="s">
         <v>40</v>
       </c>
@@ -2512,13 +2531,13 @@
       <c r="D2" s="30"/>
       <c r="E2" s="31"/>
     </row>
-    <row r="3" spans="2:8" ht="24.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" ht="24.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="32"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
       <c r="E3" s="34"/>
     </row>
-    <row r="4" spans="2:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="17" t="s">
         <v>29</v>
       </c>
@@ -2535,7 +2554,7 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="2:8" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="23" t="s">
         <v>32</v>
       </c>
@@ -2552,7 +2571,7 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="2:8" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="24"/>
       <c r="C6" s="9" t="s">
         <v>34</v>
@@ -2565,7 +2584,7 @@
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="2:8" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="24"/>
       <c r="C7" s="9" t="s">
         <v>35</v>
@@ -2576,7 +2595,7 @@
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="2:8" ht="39.450000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" ht="39.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="25"/>
       <c r="C8" s="10" t="s">
         <v>36</v>
@@ -2587,7 +2606,7 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="2:8" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="26" t="s">
         <v>37</v>
       </c>
@@ -2604,7 +2623,7 @@
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
     </row>
-    <row r="10" spans="2:8" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="27"/>
       <c r="C10" s="12" t="s">
         <v>45</v>
@@ -2615,7 +2634,7 @@
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="2:8" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="27"/>
       <c r="C11" s="12" t="s">
         <v>38</v>
@@ -2626,7 +2645,7 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="2:8" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="28"/>
       <c r="C12" s="13" t="s">
         <v>39</v>
@@ -2637,7 +2656,7 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="2:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="35" t="s">
         <v>41</v>
       </c>
@@ -2654,7 +2673,7 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="36"/>
       <c r="C14" s="15" t="s">
         <v>43</v>
@@ -2669,7 +2688,7 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" spans="2:8" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" ht="47.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B15" s="37"/>
       <c r="C15" s="16" t="s">
         <v>44</v>
@@ -2682,7 +2701,7 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2691,7 +2710,7 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -2700,7 +2719,7 @@
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -2709,7 +2728,7 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2718,7 +2737,7 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -2727,7 +2746,7 @@
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -2736,7 +2755,7 @@
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -2745,7 +2764,7 @@
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -2754,7 +2773,7 @@
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -2763,7 +2782,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -2772,7 +2791,7 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -2781,7 +2800,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -2790,7 +2809,7 @@
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -2799,7 +2818,7 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -2808,7 +2827,7 @@
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -2817,7 +2836,7 @@
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -2826,7 +2845,7 @@
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -2835,7 +2854,7 @@
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -2844,7 +2863,7 @@
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -2853,7 +2872,7 @@
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -2862,7 +2881,7 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
@@ -2871,7 +2890,7 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -2894,4 +2913,66 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A0A6A8D-49F5-4FCE-93AD-C7AEB4A44F57}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="6">
+        <f>((B2)^2*B3*B4*B1)/((B5)^2*(B1-1)+(B2)^2*B3*B4)</f>
+        <v>90.868648869147407</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>